<commit_message>
Meetings: setup asks how she records meetings and offers Copilot, Fireflies, Notion or nothing; /meetings turns a meeting into notes and tasks; Fireflies reader with her own key
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/secrets/keys.example.xlsx
+++ b/secrets/keys.example.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -467,6 +467,13 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FIREFLIES_API_KEY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Images: setup wizard for KIE.ai (sign up, credits, key moved from her clipboard into the keys file), /images skill and kie_image.py; keys.py --set
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/secrets/keys.example.xlsx
+++ b/secrets/keys.example.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -474,6 +474,13 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>KIE_API_KEY</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>